<commit_message>
Weekly golf model update
</commit_message>
<xml_diff>
--- a/golf_model.xlsx
+++ b/golf_model.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-26 22:43</t>
+          <t>2026-06-01 17:13</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9.300000000000001</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="9">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>49.7</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="10">
@@ -3594,134 +3594,134 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85.90000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="C2" t="n">
-        <v>71.40000000000001</v>
+        <v>66.3</v>
       </c>
       <c r="D2" t="n">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="E2" t="n">
-        <v>7.3</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>83.8</v>
+        <v>80</v>
       </c>
       <c r="C3" t="n">
-        <v>72</v>
+        <v>67.7</v>
       </c>
       <c r="D3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E3" t="n">
-        <v>8.1</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>89.5</v>
+        <v>80.3</v>
       </c>
       <c r="C4" t="n">
-        <v>70.3</v>
+        <v>57.8</v>
       </c>
       <c r="D4" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="E4" t="n">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>86.59999999999999</v>
+        <v>87</v>
       </c>
       <c r="C5" t="n">
-        <v>72</v>
+        <v>62.7</v>
       </c>
       <c r="D5" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>13.9</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>83.5</v>
+        <v>89.8</v>
       </c>
       <c r="C6" t="n">
-        <v>69.3</v>
+        <v>67</v>
       </c>
       <c r="D6" t="n">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>11.2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>78.7</v>
+        <v>89.2</v>
       </c>
       <c r="C7" t="n">
-        <v>61</v>
+        <v>68.8</v>
       </c>
       <c r="D7" t="n">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>11.1</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>68.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="C8" t="n">
-        <v>62.5</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>6.2</v>
+        <v>8.9</v>
       </c>
     </row>
   </sheetData>
@@ -3820,10 +3820,10 @@
         <v>95.65000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>95.5925</v>
+        <v>97.0925</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
@@ -3859,10 +3859,10 @@
         <v>93.7</v>
       </c>
       <c r="H3" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>93.765</v>
+        <v>95.265</v>
       </c>
       <c r="J3" t="n">
         <v>2</v>
@@ -3898,10 +3898,10 @@
         <v>92.69999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>92.765</v>
+        <v>94.265</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -3937,10 +3937,10 @@
         <v>92.54999999999998</v>
       </c>
       <c r="H5" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>91.7475</v>
+        <v>93.2475</v>
       </c>
       <c r="J5" t="n">
         <v>4</v>
@@ -3976,10 +3976,10 @@
         <v>90.80000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>90.41000000000001</v>
+        <v>91.91000000000001</v>
       </c>
       <c r="J6" t="n">
         <v>5</v>
@@ -4015,10 +4015,10 @@
         <v>88.7</v>
       </c>
       <c r="H7" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>88.91499999999999</v>
+        <v>90.41499999999999</v>
       </c>
       <c r="J7" t="n">
         <v>6</v>
@@ -4054,10 +4054,10 @@
         <v>89.64999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>88.7925</v>
+        <v>90.2925</v>
       </c>
       <c r="J8" t="n">
         <v>7</v>
@@ -4093,10 +4093,10 @@
         <v>87.39999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>87.23</v>
+        <v>88.73</v>
       </c>
       <c r="J9" t="n">
         <v>8</v>
@@ -4132,10 +4132,10 @@
         <v>87.84999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>86.88250000000001</v>
+        <v>88.38250000000001</v>
       </c>
       <c r="J10" t="n">
         <v>9</v>
@@ -4171,10 +4171,10 @@
         <v>87.75</v>
       </c>
       <c r="H11" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>86.6875</v>
+        <v>88.1875</v>
       </c>
       <c r="J11" t="n">
         <v>10</v>
@@ -4210,10 +4210,10 @@
         <v>86.65000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>85.64250000000001</v>
+        <v>87.14250000000001</v>
       </c>
       <c r="J12" t="n">
         <v>11</v>
@@ -4249,10 +4249,10 @@
         <v>84.95</v>
       </c>
       <c r="H13" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>84.3275</v>
+        <v>85.8275</v>
       </c>
       <c r="J13" t="n">
         <v>12</v>
@@ -4288,10 +4288,10 @@
         <v>84.45</v>
       </c>
       <c r="H14" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>83.55249999999999</v>
+        <v>85.05249999999999</v>
       </c>
       <c r="J14" t="n">
         <v>13</v>
@@ -4327,10 +4327,10 @@
         <v>83.7</v>
       </c>
       <c r="H15" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>82.515</v>
+        <v>84.015</v>
       </c>
       <c r="J15" t="n">
         <v>14</v>
@@ -4366,10 +4366,10 @@
         <v>83.3</v>
       </c>
       <c r="H16" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>82.48500000000001</v>
+        <v>83.98500000000001</v>
       </c>
       <c r="J16" t="n">
         <v>15</v>
@@ -4405,10 +4405,10 @@
         <v>82.80000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>81.41000000000001</v>
+        <v>82.91000000000001</v>
       </c>
       <c r="J17" t="n">
         <v>16</v>
@@ -4444,10 +4444,10 @@
         <v>82.19999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>81.28999999999999</v>
+        <v>82.78999999999999</v>
       </c>
       <c r="J18" t="n">
         <v>17</v>
@@ -4483,10 +4483,10 @@
         <v>83.30000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>81.08500000000001</v>
+        <v>82.58500000000001</v>
       </c>
       <c r="J19" t="n">
         <v>18</v>
@@ -4522,10 +4522,10 @@
         <v>83.05</v>
       </c>
       <c r="H20" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>80.82250000000002</v>
+        <v>82.32250000000002</v>
       </c>
       <c r="J20" t="n">
         <v>19</v>
@@ -4561,10 +4561,10 @@
         <v>82.10000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>79.845</v>
+        <v>81.345</v>
       </c>
       <c r="J21" t="n">
         <v>20</v>
@@ -4600,10 +4600,10 @@
         <v>82.25000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>79.7625</v>
+        <v>81.2625</v>
       </c>
       <c r="J22" t="n">
         <v>21</v>
@@ -4639,10 +4639,10 @@
         <v>81.40000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>78.83</v>
+        <v>80.33</v>
       </c>
       <c r="J23" t="n">
         <v>22</v>
@@ -4678,10 +4678,10 @@
         <v>81.09999999999999</v>
       </c>
       <c r="H24" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>78.545</v>
+        <v>80.045</v>
       </c>
       <c r="J24" t="n">
         <v>23</v>
@@ -4717,10 +4717,10 @@
         <v>80.45</v>
       </c>
       <c r="H25" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>77.70250000000001</v>
+        <v>79.20250000000001</v>
       </c>
       <c r="J25" t="n">
         <v>24</v>
@@ -4756,10 +4756,10 @@
         <v>80.5</v>
       </c>
       <c r="H26" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>77.575</v>
+        <v>79.075</v>
       </c>
       <c r="J26" t="n">
         <v>25</v>
@@ -4795,10 +4795,10 @@
         <v>80.65000000000001</v>
       </c>
       <c r="H27" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>77.0925</v>
+        <v>78.5925</v>
       </c>
       <c r="J27" t="n">
         <v>26</v>
@@ -4834,10 +4834,10 @@
         <v>80.25</v>
       </c>
       <c r="H28" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>76.7625</v>
+        <v>78.2625</v>
       </c>
       <c r="J28" t="n">
         <v>27</v>
@@ -4873,10 +4873,10 @@
         <v>80.75</v>
       </c>
       <c r="H29" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>76.28750000000001</v>
+        <v>77.78750000000001</v>
       </c>
       <c r="J29" t="n">
         <v>28</v>
@@ -4912,10 +4912,10 @@
         <v>79.5</v>
       </c>
       <c r="H30" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>75.875</v>
+        <v>77.375</v>
       </c>
       <c r="J30" t="n">
         <v>29</v>
@@ -4951,10 +4951,10 @@
         <v>79.10000000000001</v>
       </c>
       <c r="H31" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>74.995</v>
+        <v>76.495</v>
       </c>
       <c r="J31" t="n">
         <v>30</v>
@@ -4990,10 +4990,10 @@
         <v>78.40000000000001</v>
       </c>
       <c r="H32" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>74.53</v>
+        <v>76.03</v>
       </c>
       <c r="J32" t="n">
         <v>31</v>
@@ -5029,10 +5029,10 @@
         <v>78.7</v>
       </c>
       <c r="H33" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>74.11499999999999</v>
+        <v>75.61499999999999</v>
       </c>
       <c r="J33" t="n">
         <v>32</v>
@@ -5068,10 +5068,10 @@
         <v>78.75</v>
       </c>
       <c r="H34" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>73.9875</v>
+        <v>75.4875</v>
       </c>
       <c r="J34" t="n">
         <v>33</v>
@@ -5107,10 +5107,10 @@
         <v>78.34999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>73.1075</v>
+        <v>74.6075</v>
       </c>
       <c r="J35" t="n">
         <v>34</v>
@@ -5146,10 +5146,10 @@
         <v>77.5</v>
       </c>
       <c r="H36" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>72.875</v>
+        <v>74.375</v>
       </c>
       <c r="J36" t="n">
         <v>35</v>
@@ -5185,10 +5185,10 @@
         <v>77.5</v>
       </c>
       <c r="H37" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>72.175</v>
+        <v>73.675</v>
       </c>
       <c r="J37" t="n">
         <v>36</v>
@@ -5224,10 +5224,10 @@
         <v>76.55000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>71.59750000000001</v>
+        <v>73.09750000000001</v>
       </c>
       <c r="J38" t="n">
         <v>37</v>
@@ -5263,10 +5263,10 @@
         <v>77</v>
       </c>
       <c r="H39" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>71.25</v>
+        <v>72.75</v>
       </c>
       <c r="J39" t="n">
         <v>38</v>
@@ -5302,10 +5302,10 @@
         <v>77.10000000000001</v>
       </c>
       <c r="H40" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>71.14500000000001</v>
+        <v>72.64500000000001</v>
       </c>
       <c r="J40" t="n">
         <v>39</v>
@@ -5341,10 +5341,10 @@
         <v>76.55</v>
       </c>
       <c r="H41" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>70.3475</v>
+        <v>71.8475</v>
       </c>
       <c r="J41" t="n">
         <v>40</v>
@@ -5380,10 +5380,10 @@
         <v>75.95</v>
       </c>
       <c r="H42" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>69.92749999999999</v>
+        <v>71.42749999999999</v>
       </c>
       <c r="J42" t="n">
         <v>41</v>
@@ -5419,10 +5419,10 @@
         <v>75.25</v>
       </c>
       <c r="H43" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>69.0625</v>
+        <v>70.5625</v>
       </c>
       <c r="J43" t="n">
         <v>42</v>
@@ -5458,10 +5458,10 @@
         <v>75.25</v>
       </c>
       <c r="H44" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>68.91250000000001</v>
+        <v>70.41250000000001</v>
       </c>
       <c r="J44" t="n">
         <v>43</v>
@@ -5497,10 +5497,10 @@
         <v>76.2</v>
       </c>
       <c r="H45" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>68.64</v>
+        <v>70.14</v>
       </c>
       <c r="J45" t="n">
         <v>44</v>
@@ -5536,10 +5536,10 @@
         <v>75.2</v>
       </c>
       <c r="H46" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>68.34</v>
+        <v>69.84</v>
       </c>
       <c r="J46" t="n">
         <v>45</v>
@@ -5575,10 +5575,10 @@
         <v>75.59999999999999</v>
       </c>
       <c r="H47" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>67.81999999999999</v>
+        <v>69.31999999999999</v>
       </c>
       <c r="J47" t="n">
         <v>46</v>
@@ -5614,10 +5614,10 @@
         <v>75.95</v>
       </c>
       <c r="H48" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>67.12750000000001</v>
+        <v>68.62750000000001</v>
       </c>
       <c r="J48" t="n">
         <v>47</v>
@@ -5653,10 +5653,10 @@
         <v>74.34999999999999</v>
       </c>
       <c r="H49" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I49" t="n">
-        <v>67.1075</v>
+        <v>68.6075</v>
       </c>
       <c r="J49" t="n">
         <v>48</v>
@@ -5692,10 +5692,10 @@
         <v>75.05</v>
       </c>
       <c r="H50" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
-        <v>66.8725</v>
+        <v>68.3725</v>
       </c>
       <c r="J50" t="n">
         <v>49</v>
@@ -5731,10 +5731,10 @@
         <v>74.65000000000001</v>
       </c>
       <c r="H51" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>65.8425</v>
+        <v>67.3425</v>
       </c>
       <c r="J51" t="n">
         <v>50</v>
@@ -5770,10 +5770,10 @@
         <v>74.25</v>
       </c>
       <c r="H52" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>65.8125</v>
+        <v>67.3125</v>
       </c>
       <c r="J52" t="n">
         <v>51</v>
@@ -5809,10 +5809,10 @@
         <v>74.7</v>
       </c>
       <c r="H53" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>65.16500000000001</v>
+        <v>66.66500000000001</v>
       </c>
       <c r="J53" t="n">
         <v>52</v>
@@ -5848,10 +5848,10 @@
         <v>75.60000000000001</v>
       </c>
       <c r="H54" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>64.87</v>
+        <v>66.37</v>
       </c>
       <c r="J54" t="n">
         <v>53</v>
@@ -5887,10 +5887,10 @@
         <v>72.75</v>
       </c>
       <c r="H55" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>64.4375</v>
+        <v>65.9375</v>
       </c>
       <c r="J55" t="n">
         <v>54</v>
@@ -5926,10 +5926,10 @@
         <v>72.94999999999999</v>
       </c>
       <c r="H56" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>63.8275</v>
+        <v>65.3275</v>
       </c>
       <c r="J56" t="n">
         <v>55</v>
@@ -5965,10 +5965,10 @@
         <v>74.25</v>
       </c>
       <c r="H57" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>63.71250000000001</v>
+        <v>65.21250000000001</v>
       </c>
       <c r="J57" t="n">
         <v>56</v>
@@ -6004,10 +6004,10 @@
         <v>74.15000000000001</v>
       </c>
       <c r="H58" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>63.51750000000001</v>
+        <v>65.01750000000001</v>
       </c>
       <c r="J58" t="n">
         <v>57</v>
@@ -6043,10 +6043,10 @@
         <v>73.90000000000001</v>
       </c>
       <c r="H59" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>62.70500000000001</v>
+        <v>64.20500000000001</v>
       </c>
       <c r="J59" t="n">
         <v>58</v>
@@ -6082,10 +6082,10 @@
         <v>74.40000000000001</v>
       </c>
       <c r="H60" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I60" t="n">
-        <v>62.38000000000001</v>
+        <v>63.88000000000001</v>
       </c>
       <c r="J60" t="n">
         <v>59</v>
@@ -6121,10 +6121,10 @@
         <v>71.8</v>
       </c>
       <c r="H61" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
-        <v>61.91</v>
+        <v>63.41</v>
       </c>
       <c r="J61" t="n">
         <v>60</v>

</xml_diff>